<commit_message>
update new specimens on morphosource
</commit_message>
<xml_diff>
--- a/Volume_and_morphosource_ID.xlsx
+++ b/Volume_and_morphosource_ID.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Document_UQAR\These\chapitre_1\Article\projet_git_hub\Raw_data_Axolotl_Brains\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A375F62-E8A5-40CD-B414-98C05042C2A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55DDA013-C1DE-47F7-B841-1F1AF41FDD29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuille 1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="228">
   <si>
     <t>ID</t>
   </si>
@@ -682,6 +682,33 @@
   </si>
   <si>
     <t>000786641</t>
+  </si>
+  <si>
+    <t>000857180</t>
+  </si>
+  <si>
+    <t>000857185</t>
+  </si>
+  <si>
+    <t>000857190</t>
+  </si>
+  <si>
+    <t>000857195</t>
+  </si>
+  <si>
+    <t>000857201</t>
+  </si>
+  <si>
+    <t>000857206</t>
+  </si>
+  <si>
+    <t>000857217</t>
+  </si>
+  <si>
+    <t>000857222</t>
+  </si>
+  <si>
+    <t>000857227</t>
   </si>
 </sst>
 </file>
@@ -2737,6 +2764,9 @@
       <c r="L42" s="4">
         <v>0.40007983349999998</v>
       </c>
+      <c r="M42" s="7" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="43" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
@@ -2802,6 +2832,9 @@
       <c r="L44" s="4">
         <v>0.52539216990000004</v>
       </c>
+      <c r="M44" s="7" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="45" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
@@ -2840,6 +2873,9 @@
       <c r="L45" s="4">
         <v>0.54321463380000001</v>
       </c>
+      <c r="M45" s="7" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="46" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
@@ -2878,6 +2914,9 @@
       <c r="L46" s="4">
         <v>0.40637066170000002</v>
       </c>
+      <c r="M46" s="7" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="47" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
@@ -2916,6 +2955,9 @@
       <c r="L47" s="4">
         <v>0.489282936</v>
       </c>
+      <c r="M47" s="7" t="s">
+        <v>223</v>
+      </c>
     </row>
     <row r="48" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
@@ -2954,6 +2996,9 @@
       <c r="L48" s="4">
         <v>0.36909546710000002</v>
       </c>
+      <c r="M48" s="7" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="49" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
@@ -2992,6 +3037,9 @@
       <c r="L49" s="4">
         <v>0.4858621648</v>
       </c>
+      <c r="M49" s="7" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="50" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
@@ -3030,6 +3078,9 @@
       <c r="L50" s="4">
         <v>0.45069029329999999</v>
       </c>
+      <c r="M50" s="7" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="51" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
@@ -3067,6 +3118,9 @@
       </c>
       <c r="L51" s="4">
         <v>0.40886664890000002</v>
+      </c>
+      <c r="M51" s="7" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="52" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
New specimens on morphosource
</commit_message>
<xml_diff>
--- a/Volume_and_morphosource_ID.xlsx
+++ b/Volume_and_morphosource_ID.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Document_UQAR\These\chapitre_1\Article\projet_git_hub\Raw_data_Axolotl_Brains\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55DDA013-C1DE-47F7-B841-1F1AF41FDD29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97B10AD0-9A2B-489C-8C69-75AE30F9D662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="237">
   <si>
     <t>ID</t>
   </si>
@@ -709,6 +709,33 @@
   </si>
   <si>
     <t>000857227</t>
+  </si>
+  <si>
+    <t>000859280</t>
+  </si>
+  <si>
+    <t>000859288</t>
+  </si>
+  <si>
+    <t>000859289</t>
+  </si>
+  <si>
+    <t>000859297</t>
+  </si>
+  <si>
+    <t>000859304</t>
+  </si>
+  <si>
+    <t>000859309</t>
+  </si>
+  <si>
+    <t>000859314</t>
+  </si>
+  <si>
+    <t>000859319</t>
+  </si>
+  <si>
+    <t>000859324</t>
   </si>
 </sst>
 </file>
@@ -3187,6 +3214,9 @@
       <c r="L53" s="4">
         <v>0.44422282089999998</v>
       </c>
+      <c r="M53" s="7" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="54" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
@@ -3225,6 +3255,9 @@
       <c r="L54" s="4">
         <v>0.49070757370000001</v>
       </c>
+      <c r="M54" s="7" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="55" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
@@ -3263,6 +3296,9 @@
       <c r="L55" s="4">
         <v>0.45674431999999998</v>
       </c>
+      <c r="M55" s="7" t="s">
+        <v>230</v>
+      </c>
     </row>
     <row r="56" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
@@ -3301,6 +3337,9 @@
       <c r="L56" s="4">
         <v>0.46049650399999997</v>
       </c>
+      <c r="M56" s="7" t="s">
+        <v>231</v>
+      </c>
     </row>
     <row r="57" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
@@ -3339,6 +3378,9 @@
       <c r="L57" s="4">
         <v>0.40912641970000002</v>
       </c>
+      <c r="M57" s="7" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="58" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
@@ -3377,6 +3419,9 @@
       <c r="L58" s="4">
         <v>0.4274536592</v>
       </c>
+      <c r="M58" s="7" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="59" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
@@ -3415,6 +3460,9 @@
       <c r="L59" s="4">
         <v>0.50195154740000003</v>
       </c>
+      <c r="M59" s="7" t="s">
+        <v>234</v>
+      </c>
     </row>
     <row r="60" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
@@ -3453,6 +3501,9 @@
       <c r="L60" s="4">
         <v>0.378718471</v>
       </c>
+      <c r="M60" s="7" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="61" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
@@ -3490,6 +3541,9 @@
       </c>
       <c r="L61" s="4">
         <v>0.41869364120000002</v>
+      </c>
+      <c r="M61" s="7" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="62" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
all specimens added to morphosource
</commit_message>
<xml_diff>
--- a/Volume_and_morphosource_ID.xlsx
+++ b/Volume_and_morphosource_ID.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Document_UQAR\These\chapitre_1\Article\projet_git_hub\Raw_data_Axolotl_Brains\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97B10AD0-9A2B-489C-8C69-75AE30F9D662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E58BF22F-8C4D-416A-BDF6-6BD1C8CD8FC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="257">
   <si>
     <t>ID</t>
   </si>
@@ -736,6 +736,66 @@
   </si>
   <si>
     <t>000859324</t>
+  </si>
+  <si>
+    <t>000859336</t>
+  </si>
+  <si>
+    <t>000859341</t>
+  </si>
+  <si>
+    <t>000859346</t>
+  </si>
+  <si>
+    <t>000859352</t>
+  </si>
+  <si>
+    <t>000859356</t>
+  </si>
+  <si>
+    <t>000859364</t>
+  </si>
+  <si>
+    <t>000859370</t>
+  </si>
+  <si>
+    <t>000859373</t>
+  </si>
+  <si>
+    <t>000859379</t>
+  </si>
+  <si>
+    <t>000859384</t>
+  </si>
+  <si>
+    <t>000859648</t>
+  </si>
+  <si>
+    <t>000859649</t>
+  </si>
+  <si>
+    <t>000859650</t>
+  </si>
+  <si>
+    <t>000859657</t>
+  </si>
+  <si>
+    <t>000859662</t>
+  </si>
+  <si>
+    <t>000859667</t>
+  </si>
+  <si>
+    <t>000859675</t>
+  </si>
+  <si>
+    <t>000859676</t>
+  </si>
+  <si>
+    <t>000859682</t>
+  </si>
+  <si>
+    <t>000859687</t>
   </si>
 </sst>
 </file>
@@ -3583,6 +3643,9 @@
       <c r="L62" s="4">
         <v>0.57481916879999995</v>
       </c>
+      <c r="M62" s="7" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="63" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
@@ -3621,6 +3684,9 @@
       <c r="L63" s="4">
         <v>0.43637719609999998</v>
       </c>
+      <c r="M63" s="7" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="64" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
@@ -3659,8 +3725,11 @@
       <c r="L64" s="4">
         <v>0.4617537947</v>
       </c>
-    </row>
-    <row r="65" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M64" s="7" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>65</v>
       </c>
@@ -3697,8 +3766,11 @@
       <c r="L65" s="4">
         <v>0.52310071810000003</v>
       </c>
-    </row>
-    <row r="66" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M65" s="7" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>66</v>
       </c>
@@ -3735,8 +3807,11 @@
       <c r="L66" s="4">
         <v>0.45774019919999998</v>
       </c>
-    </row>
-    <row r="67" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M66" s="7" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>67</v>
       </c>
@@ -3773,8 +3848,11 @@
       <c r="L67" s="4">
         <v>0.54832856370000005</v>
       </c>
-    </row>
-    <row r="68" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M67" s="7" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>68</v>
       </c>
@@ -3811,8 +3889,11 @@
       <c r="L68" s="4">
         <v>0.47296112699999998</v>
       </c>
-    </row>
-    <row r="69" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M68" s="7" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>69</v>
       </c>
@@ -3849,8 +3930,11 @@
       <c r="L69" s="4">
         <v>0.49193150429999999</v>
       </c>
-    </row>
-    <row r="70" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M69" s="7" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>70</v>
       </c>
@@ -3887,8 +3971,11 @@
       <c r="L70" s="4">
         <v>0.54727143330000005</v>
       </c>
-    </row>
-    <row r="71" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M70" s="7" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>71</v>
       </c>
@@ -3925,8 +4012,11 @@
       <c r="L71" s="4">
         <v>0.55508205740000005</v>
       </c>
-    </row>
-    <row r="72" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M71" s="7" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>72</v>
       </c>
@@ -3963,8 +4053,11 @@
       <c r="L72" s="4">
         <v>0.39515348550000001</v>
       </c>
-    </row>
-    <row r="73" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M72" s="7" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>73</v>
       </c>
@@ -4001,8 +4094,11 @@
       <c r="L73" s="4">
         <v>0.61944450959999997</v>
       </c>
-    </row>
-    <row r="74" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M73" s="7" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>74</v>
       </c>
@@ -4039,8 +4135,11 @@
       <c r="L74" s="4">
         <v>0.50836159680000004</v>
       </c>
-    </row>
-    <row r="75" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M74" s="7" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>75</v>
       </c>
@@ -4077,8 +4176,11 @@
       <c r="L75" s="4">
         <v>0.53472696500000005</v>
       </c>
-    </row>
-    <row r="76" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M75" s="7" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>76</v>
       </c>
@@ -4115,8 +4217,11 @@
       <c r="L76" s="4">
         <v>0.53130619379999999</v>
       </c>
-    </row>
-    <row r="77" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M76" s="7" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>77</v>
       </c>
@@ -4153,8 +4258,11 @@
       <c r="L77" s="4">
         <v>0.51756459239999997</v>
       </c>
-    </row>
-    <row r="78" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M77" s="7" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>78</v>
       </c>
@@ -4191,8 +4299,11 @@
       <c r="L78" s="4">
         <v>0.4853349669</v>
       </c>
-    </row>
-    <row r="79" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M78" s="7" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="79" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>79</v>
       </c>
@@ -4229,8 +4340,11 @@
       <c r="L79" s="4">
         <v>0.41869528189999999</v>
       </c>
-    </row>
-    <row r="80" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M79" s="7" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>80</v>
       </c>
@@ -4266,6 +4380,9 @@
       </c>
       <c r="L80" s="4">
         <v>0.53708896510000004</v>
+      </c>
+      <c r="M80" s="7" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="81" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -4304,6 +4421,9 @@
       </c>
       <c r="L81" s="4">
         <v>0.31413398320000002</v>
+      </c>
+      <c r="M81" s="7" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="82" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">

</xml_diff>